<commit_message>
Restrukturisasi alur KDD, model komparasi, dan visualisasi
</commit_message>
<xml_diff>
--- a/tahap3_hasil_baseline.xlsx
+++ b/tahap3_hasil_baseline.xlsx
@@ -425,215 +425,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Dataset</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Filters</t>
+          <t>Baris Asli</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Kernel</t>
+          <t>Window Size</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Units</t>
+          <t>Dimensi 3D Input (Samples, Window, Features)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Dropout</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Window</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Batch</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>MSE</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>MAE</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>RMSE</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>MAPE</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>R2</t>
+          <t>Dimensi Target Output</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CNN Saja (Tanpa Optimasi)</t>
+          <t>Data Pelatihan (Train)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64</v>
+        <v>2566</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>(2536, 30, 6)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>30</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="H2" t="n">
-        <v>32</v>
-      </c>
-      <c r="I2" t="n">
-        <v>11127.6917</v>
-      </c>
-      <c r="J2" t="n">
-        <v>84.3831</v>
-      </c>
-      <c r="K2" t="n">
-        <v>105.4879</v>
-      </c>
-      <c r="L2" t="n">
-        <v>2.9247</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.9026999999999999</v>
+          <t>(2536,)</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LSTM Saja (Tanpa Optimasi)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>64</v>
+          <t>Data Pengujian (Test)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>642</v>
+      </c>
+      <c r="C3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>(612, 30, 6)</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>30</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="H3" t="n">
-        <v>32</v>
-      </c>
-      <c r="I3" t="n">
-        <v>6036.1562</v>
-      </c>
-      <c r="J3" t="n">
-        <v>62.2869</v>
-      </c>
-      <c r="K3" t="n">
-        <v>77.6927</v>
-      </c>
-      <c r="L3" t="n">
-        <v>2.1782</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.9472</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CNN-LSTM (Tanpa Optimasi)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>64</v>
-      </c>
-      <c r="C4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" t="n">
-        <v>64</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>30</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="H4" t="n">
-        <v>32</v>
-      </c>
-      <c r="I4" t="n">
-        <v>5012.4793</v>
-      </c>
-      <c r="J4" t="n">
-        <v>56.2661</v>
-      </c>
-      <c r="K4" t="n">
-        <v>70.7989</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1.9414</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.9562</v>
+          <t>(612,)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>